<commit_message>
feat(templates): upgrade official 出厂底价表 and dual-sheet public templates to flagship version
</commit_message>
<xml_diff>
--- a/public/templates/极简出厂底价表_双表旗舰版.xlsx
+++ b/public/templates/极简出厂底价表_双表旗舰版.xlsx
@@ -4,15 +4,59 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="⚙️ 全局核算参数 (Config)" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="📦 商品出厂底价库 (Products)" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="📌 使用指南与提效神器" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="⚙️ 全局核算参数 (Config)" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="📦 商品出厂底价库 (Products)" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="📄 对外纯净批量报价单 (脱敏单)" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="162">
+  <si>
+    <t>【2026 外贸出厂核算控制台与批量算价神表 · Kelvin旗舰版】使用指南</t>
+  </si>
+  <si>
+    <t>💡 本地离线版与线上版 KelvinFlow (https://quote.kelvinflow.com) 采用 100% 相同数据架构。在此填写的全部数据，日后可直接无损上传，零学习成本。</t>
+  </si>
+  <si>
+    <t>1. 为什么做这套表？</t>
+  </si>
+  <si>
+    <t>拒绝单品手工反复按计算器！本表专为工贸一体外贸工厂、外贸公司与独立业务员打造。左侧批量录入底价与箱规，右侧全自动联动秒出全量多币种 FOB 美金单价、集装箱装柜量与利润红线防御。</t>
+  </si>
+  <si>
+    <t>2. 【⚙️ 全局核算参数】怎么用？</t>
+  </si>
+  <si>
+    <t>在第 2 张工作表设定贵司的内部锁定汇率（如 USD 7.20）、全厂保底毛利（如 15%）、利润防穿底红线（如 8%）与海运进仓港杂平摊（如 0.20 元/件）。在此修改后，全厂全量商品自动秒级联动更新。</t>
+  </si>
+  <si>
+    <t>3. 【📦 商品出厂底价库】怎么用？</t>
+  </si>
+  <si>
+    <t>在第 3 张工作表批量录入产品 SKU、出厂底价与包装尺寸。黄色公式区会自动联动倒算出精准 FOB 美金报价、自动算出 20GP/40HQ 可装柜件数；若某品毛利低于红线会自动闪烁警报。</t>
+  </si>
+  <si>
+    <t>4. 对外发给买家安全吗？</t>
+  </si>
+  <si>
+    <t>100% 安全！第 4 张工作表【📄 对外纯净批量报价单】专为海外买家设计，工厂出厂底价、内部成本与真实毛利率全部自动脱敏隐藏，可直接打印或导出 PDF 发给海外买家。</t>
+  </si>
+  <si>
+    <t>5. 🚀 无缝升级线上版 (SaaS 原生直通)</t>
+  </si>
+  <si>
+    <t>本表格式与 KelvinFlow 智能出单引擎 (https://quote.kelvinflow.com) 完全一致！平时直接当离线底价库用；一旦买家发来几十个型号的长篇英文邮件或 PDF 询盘，直接把本表上传到系统，转发邮件，AI 10 秒自动审单对齐底价生成专业英文报价单。小红书官方群友免审开通 7 天深度体验。</t>
+  </si>
+  <si>
+    <t>6. 开源与版权说明</t>
+  </si>
+  <si>
+    <t>由大湾区全栈独立开发者 Kelvin (IT佬Kelvin) 荣誉出品，永久免费，纯净无广告，禁止二次倒卖。欢迎在小红书官方粉丝群内交流探讨！</t>
+  </si>
   <si>
     <t>🏢 我司外贸出厂核算控制台 · 全局业务参数配置 (Global Configuration)</t>
   </si>
@@ -110,9 +154,6 @@
     <t>全厂默认保底毛利率 (Default Margin)</t>
   </si>
   <si>
-    <t>15%</t>
-  </si>
-  <si>
     <t>百分比 (0.15)</t>
   </si>
   <si>
@@ -125,9 +166,6 @@
     <t>最低保护红线毛利率 (Floor Margin)</t>
   </si>
   <si>
-    <t>8%</t>
-  </si>
-  <si>
     <t>百分比 (0.08)</t>
   </si>
   <si>
@@ -140,9 +178,6 @@
     <t>样品打样费上浮倍率 (Sample Multiplier)</t>
   </si>
   <si>
-    <t>2.5</t>
-  </si>
-  <si>
     <t>倍率 (出厂价*2.5)</t>
   </si>
   <si>
@@ -191,9 +226,6 @@
     <t>工厂车间自提 (Factory Ex-works)</t>
   </si>
   <si>
-    <t>¥0.00</t>
-  </si>
-  <si>
     <t>买家自提，仅含标准纸箱包装，无港口杂费与拖车费</t>
   </si>
   <si>
@@ -203,12 +235,6 @@
     <t>深圳盐田港 / 蛇口港 (Shenzhen)</t>
   </si>
   <si>
-    <t>¥0.20</t>
-  </si>
-  <si>
-    <t>¥1,500.00</t>
-  </si>
-  <si>
     <t>包含工厂至深圳码头内陆拖车、出口报关、港杂码头费(THC)</t>
   </si>
   <si>
@@ -248,9 +274,6 @@
     <t>100% T/T Advance (全款预付)</t>
   </si>
   <si>
-    <t>-2.0% (直享折扣)</t>
-  </si>
-  <si>
     <t>USD / EUR / GBP</t>
   </si>
   <si>
@@ -263,9 +286,6 @@
     <t>30% Deposit + 70% Balance (标准前T/T)</t>
   </si>
   <si>
-    <t>0.0% (基准价格)</t>
-  </si>
-  <si>
     <t>外贸行业标准条款：30%定金排产，70%见提单副本付款</t>
   </si>
   <si>
@@ -275,9 +295,6 @@
     <t>L/C at Sight (即期不可撤销信用证)</t>
   </si>
   <si>
-    <t>+1.5% (微幅上浮)</t>
-  </si>
-  <si>
     <t>USD / EUR</t>
   </si>
   <si>
@@ -308,42 +325,18 @@
     <t>20GP (20尺小柜)</t>
   </si>
   <si>
-    <t>28.0 CBM</t>
-  </si>
-  <si>
-    <t>33.2 CBM</t>
-  </si>
-  <si>
-    <t>21,800 KG</t>
-  </si>
-  <si>
     <t>适合五金紧固件、金属椅脚等高密度重货或试单</t>
   </si>
   <si>
     <t>40GP (40尺平柜)</t>
   </si>
   <si>
-    <t>58.0 CBM</t>
-  </si>
-  <si>
-    <t>67.7 CBM</t>
-  </si>
-  <si>
-    <t>26,000 KG</t>
-  </si>
-  <si>
     <t>适合体积适中、重量适中的常规工业品与配件</t>
   </si>
   <si>
     <t>40HQ (40尺高柜)</t>
   </si>
   <si>
-    <t>68.0 CBM</t>
-  </si>
-  <si>
-    <t>76.3 CBM</t>
-  </si>
-  <si>
     <t>适合办公椅、支架、轻泡货等大体积外贸商品</t>
   </si>
   <si>
@@ -380,6 +373,24 @@
     <t>海关编码 HS Code (选填)</t>
   </si>
   <si>
+    <t>⚡ 单件港杂平摊(RMB)</t>
+  </si>
+  <si>
+    <t>⚡ 生效核算毛利率</t>
+  </si>
+  <si>
+    <t>🎯 FOB美金单价(USD)</t>
+  </si>
+  <si>
+    <t>📦 20GP小柜装量(PCS)</t>
+  </si>
+  <si>
+    <t>📦 40HQ高柜装量(PCS)</t>
+  </si>
+  <si>
+    <t>🛡️ 利润安全状态</t>
+  </si>
+  <si>
     <t>ST-2026-A</t>
   </si>
   <si>
@@ -389,9 +400,6 @@
     <t>Aluminum Alloy Precision Bracket (铝合金精密五金支架)</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>20-25 Days</t>
   </si>
   <si>
@@ -407,9 +415,6 @@
     <t>Stainless Steel Hex Fastener Screws (不锈钢沉头紧固件螺丝)</t>
   </si>
   <si>
-    <t>18%</t>
-  </si>
-  <si>
     <t>15-20 Days</t>
   </si>
   <si>
@@ -425,9 +430,6 @@
     <t>Ergonomic Mesh Office Chair (高档网布人体工学办公椅)</t>
   </si>
   <si>
-    <t>25%</t>
-  </si>
-  <si>
     <t>30-35 Days</t>
   </si>
   <si>
@@ -462,16 +464,59 @@
   </si>
   <si>
     <t>3D Armrest Pro, PU Armrest Plus, 加强升降扶手, ARM-09</t>
+  </si>
+  <si>
+    <t>GLOBAL EXPORT FORMAL QUOTATION (COMMERCIAL OFFER)</t>
+  </si>
+  <si>
+    <t>Trade Term: FOB Shenzhen (Incoterms 2020)  |  Currency: USD ($)</t>
+  </si>
+  <si>
+    <t>Payment: 30% Deposit, 70% Before Shipment  |  Price Validity: 30 Days</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Model No.</t>
+  </si>
+  <si>
+    <t>Product Description &amp; Detailed Specifications</t>
+  </si>
+  <si>
+    <t>MOQ (PCS)</t>
+  </si>
+  <si>
+    <t>FOB Price (USD)</t>
+  </si>
+  <si>
+    <t>Packing (PCS/CTN)</t>
+  </si>
+  <si>
+    <t>20GP Est. (PCS)</t>
+  </si>
+  <si>
+    <t>40HQ Est. (PCS)</t>
+  </si>
+  <si>
+    <t>Lead Time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="¥#,##0.00"/>
+  <numFmts count="8">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="¥#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot; CBM&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0&quot; KG&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -481,52 +526,115 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="13"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
-      <color rgb="475569"/>
+      <i/>
+      <color rgb="FF475569"/>
       <sz val="9.5"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <color rgb="1E3A8A"/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="10"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="9.5"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A8A"/>
       <sz val="11"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <color rgb="1E293B"/>
+      <color rgb="FF1E293B"/>
       <sz val="10"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
-      <color rgb="1E293B"/>
+      <color rgb="FF1E293B"/>
       <sz val="10"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
+      <color rgb="FFB91C1C"/>
+      <sz val="10"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <color rgb="FFB91C1C"/>
+      <sz val="10"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10.5"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <color rgb="B91C1C"/>
-      <sz val="10"/>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
       <name val="Microsoft YaHei"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="9.5"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,22 +643,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1E3A8A"/>
+        <fgColor rgb="FF1E3A8A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F8FAFC"/>
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="DBEAFE"/>
+        <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="2563EB"/>
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2563EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD97706"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -564,16 +687,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -581,45 +704,201 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -961,469 +1240,548 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:C10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="85" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="5" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
-    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="5" max="5" width="54" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="5">
+    <row r="2" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="4" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="10">
         <v>7.2</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="8">
+      <c r="C6" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="14">
         <v>7.85</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="C7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="10">
         <v>9.1</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="8">
+      <c r="C8" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="14">
         <v>4.8</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="5">
+      <c r="C9" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="10">
         <v>5.3</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-    </row>
-    <row r="13" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="C10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="9" t="s">
+      <c r="E10" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="10" t="s">
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="B13" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C13" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D13" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="7" t="s">
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="B14" s="18">
+        <v>0.15</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="D14" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="E14" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="10" t="s">
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="B15" s="20">
+        <v>0.08</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+      <c r="D15" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-    </row>
-    <row r="20" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="E15" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="4" t="s">
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="B16" s="23">
+        <v>2.5</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D16" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E16" s="12" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+    <row r="17" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B17" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C17" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="7" t="s">
+      <c r="D17" s="16" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="22" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="E17" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="9" t="s">
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="B20" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="C20" s="8" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="D20" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="E20" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="6" t="s">
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="B21" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="C21" s="25">
+        <v>0</v>
+      </c>
+      <c r="D21" s="25">
+        <v>0</v>
+      </c>
+      <c r="E21" s="12" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-    </row>
-    <row r="26" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="B22" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C22" s="26">
+        <v>0.2</v>
+      </c>
+      <c r="D22" s="26">
+        <v>1500</v>
+      </c>
+      <c r="E22" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="4" t="s">
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="B23" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="C23" s="11" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="27" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="D23" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="E23" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="6" t="s">
+    </row>
+    <row r="25" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="B26" s="8" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="28" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+      <c r="C26" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="D26" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="10" t="s">
+      <c r="E26" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E28" s="10" t="s">
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="29" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="B27" s="27">
+        <v>-0.02</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="D27" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="E27" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="7" t="s">
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="B28" s="28">
+        <v>0</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="16" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="31" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+      <c r="E28" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-    </row>
-    <row r="32" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B29" s="27">
+        <v>0.015</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="D29" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="E29" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="E32" s="4" t="s">
+    </row>
+    <row r="31" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="33" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B32" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C32" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D32" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E32" s="8" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
+    <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B33" s="29">
+        <v>28</v>
+      </c>
+      <c r="C33" s="29">
+        <v>33.2</v>
+      </c>
+      <c r="D33" s="30">
+        <v>21800</v>
+      </c>
+      <c r="E33" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="C34" s="9" t="s">
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="B34" s="31">
+        <v>58</v>
+      </c>
+      <c r="C34" s="31">
+        <v>67.7</v>
+      </c>
+      <c r="D34" s="32">
+        <v>26000</v>
+      </c>
+      <c r="E34" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="E34" s="10" t="s">
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="35" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
+      <c r="B35" s="29">
+        <v>68</v>
+      </c>
+      <c r="C35" s="29">
+        <v>76.3</v>
+      </c>
+      <c r="D35" s="30">
+        <v>26000</v>
+      </c>
+      <c r="E35" s="12" t="s">
         <v>107</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1441,269 +1799,648 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="65" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
-    <col min="9" max="10" width="38" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="2" max="2" width="55" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="10" width="36" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="25" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="28" customWidth="1"/>
+    <col min="15" max="16" width="26" customWidth="1"/>
+    <col min="17" max="17" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="E1" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="F1" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="G1" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="H1" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="I1" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="J1" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="K1" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="L1" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="M1" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="N1" s="34" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="O1" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="P1" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="Q1" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="12">
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="37">
         <v>15.5</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="38">
         <v>500</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="38">
         <v>50</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="39">
         <v>0.045</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="40">
         <v>14.5</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="I2" s="41"/>
+      <c r="J2" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="K2" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="L2" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M2" s="43">
+        <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$14, I2)</f>
+      </c>
+      <c r="N2" s="44">
+        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O2" s="45">
+        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G2)) * F2, "-")</f>
+      </c>
+      <c r="P2" s="45">
+        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G2)) * F2, "-")</f>
+      </c>
+      <c r="Q2" s="46">
+        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="47" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="13">
+      <c r="B3" s="48" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="49">
         <v>0.85</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="50">
         <v>5000</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="50">
         <v>1000</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="51">
         <v>0.02</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="52">
         <v>18</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="K3" s="9" t="s">
+      <c r="I3" s="53">
+        <v>0.18</v>
+      </c>
+      <c r="J3" s="47" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="4" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="K3" s="47" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="L3" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M3" s="43">
+        <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$14, I3)</f>
+      </c>
+      <c r="N3" s="44">
+        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O3" s="45">
+        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G3)) * F3, "-")</f>
+      </c>
+      <c r="P3" s="45">
+        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G3)) * F3, "-")</f>
+      </c>
+      <c r="Q3" s="46">
+        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="D4" s="12">
+      <c r="C4" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="37">
         <v>185</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="38">
         <v>50</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="38">
         <v>1</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="39">
         <v>0.16</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="40">
         <v>16.2</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="I4" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="J4" s="35" t="s">
         <v>138</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="35" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="5" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="L4" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M4" s="43">
+        <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$14, I4)</f>
+      </c>
+      <c r="N4" s="44">
+        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O4" s="45">
+        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G4)) * F4, "-")</f>
+      </c>
+      <c r="P4" s="45">
+        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G4)) * F4, "-")</f>
+      </c>
+      <c r="Q4" s="46">
+        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="48" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="49">
         <v>38</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="50">
         <v>200</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="50">
         <v>5</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="51">
         <v>0.08</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="52">
         <v>11</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="J5" s="9" t="s">
+      <c r="I5" s="53"/>
+      <c r="J5" s="47" t="s">
         <v>143</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="K5" s="47" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="6" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="L5" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M5" s="43">
+        <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$14, I5)</f>
+      </c>
+      <c r="N5" s="44">
+        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O5" s="45">
+        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G5)) * F5, "-")</f>
+      </c>
+      <c r="P5" s="45">
+        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G5)) * F5, "-")</f>
+      </c>
+      <c r="Q5" s="46">
+        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="36" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="36" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="37">
         <v>24</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="38">
         <v>300</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="38">
         <v>20</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="39">
         <v>0.055</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="40">
         <v>9.5</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="K6" s="6" t="s">
+      <c r="I6" s="41"/>
+      <c r="J6" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="K6" s="35" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="7" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="L6" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M6" s="43">
+        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$14, I6)</f>
+      </c>
+      <c r="N6" s="44">
+        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O6" s="45">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G6)) * F6, "-")</f>
+      </c>
+      <c r="P6" s="45">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G6)) * F6, "-")</f>
+      </c>
+      <c r="Q6" s="46">
+        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="47" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="49">
         <v>25</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="50">
         <v>300</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="50">
         <v>20</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="51">
         <v>0.055</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="52">
         <v>9.5</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="K7" s="9" t="s">
+      <c r="I7" s="53"/>
+      <c r="J7" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="K7" s="47" t="s">
         <v>144</v>
+      </c>
+      <c r="L7" s="42">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
+      </c>
+      <c r="M7" s="43">
+        <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$14, I7)</f>
+      </c>
+      <c r="N7" s="44">
+        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
+      </c>
+      <c r="O7" s="45">
+        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G7)) * F7, "-")</f>
+      </c>
+      <c r="P7" s="45">
+        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G7)) * F7, "-")</f>
+      </c>
+      <c r="Q7" s="46">
+        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="9" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="54" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="55" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="56" t="s">
+        <v>152</v>
+      </c>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="57" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="57" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="57" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3" s="57" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" s="57" t="s">
+        <v>159</v>
+      </c>
+      <c r="H3" s="57" t="s">
+        <v>160</v>
+      </c>
+      <c r="I3" s="57" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="58">
+        <v>1</v>
+      </c>
+      <c r="B4" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!A2</f>
+      </c>
+      <c r="C4" s="59">
+        <f>'📦 商品出厂底价库 (Products)'!C2</f>
+      </c>
+      <c r="D4" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!E2</f>
+      </c>
+      <c r="E4" s="61">
+        <f>'📦 商品出厂底价库 (Products)'!N2</f>
+      </c>
+      <c r="F4" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!F2</f>
+      </c>
+      <c r="G4" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!O2</f>
+      </c>
+      <c r="H4" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!P2</f>
+      </c>
+      <c r="I4" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!J2</f>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="62">
+        <v>2</v>
+      </c>
+      <c r="B5" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!A3</f>
+      </c>
+      <c r="C5" s="63">
+        <f>'📦 商品出厂底价库 (Products)'!C3</f>
+      </c>
+      <c r="D5" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!E3</f>
+      </c>
+      <c r="E5" s="65">
+        <f>'📦 商品出厂底价库 (Products)'!N3</f>
+      </c>
+      <c r="F5" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!F3</f>
+      </c>
+      <c r="G5" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!O3</f>
+      </c>
+      <c r="H5" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!P3</f>
+      </c>
+      <c r="I5" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!J3</f>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="58">
+        <v>3</v>
+      </c>
+      <c r="B6" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!A4</f>
+      </c>
+      <c r="C6" s="59">
+        <f>'📦 商品出厂底价库 (Products)'!C4</f>
+      </c>
+      <c r="D6" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!E4</f>
+      </c>
+      <c r="E6" s="61">
+        <f>'📦 商品出厂底价库 (Products)'!N4</f>
+      </c>
+      <c r="F6" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!F4</f>
+      </c>
+      <c r="G6" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!O4</f>
+      </c>
+      <c r="H6" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!P4</f>
+      </c>
+      <c r="I6" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!J4</f>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="62">
+        <v>4</v>
+      </c>
+      <c r="B7" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!A5</f>
+      </c>
+      <c r="C7" s="63">
+        <f>'📦 商品出厂底价库 (Products)'!C5</f>
+      </c>
+      <c r="D7" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!E5</f>
+      </c>
+      <c r="E7" s="65">
+        <f>'📦 商品出厂底价库 (Products)'!N5</f>
+      </c>
+      <c r="F7" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!F5</f>
+      </c>
+      <c r="G7" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!O5</f>
+      </c>
+      <c r="H7" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!P5</f>
+      </c>
+      <c r="I7" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!J5</f>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="58">
+        <v>5</v>
+      </c>
+      <c r="B8" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!A6</f>
+      </c>
+      <c r="C8" s="59">
+        <f>'📦 商品出厂底价库 (Products)'!C6</f>
+      </c>
+      <c r="D8" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!E6</f>
+      </c>
+      <c r="E8" s="61">
+        <f>'📦 商品出厂底价库 (Products)'!N6</f>
+      </c>
+      <c r="F8" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!F6</f>
+      </c>
+      <c r="G8" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!O6</f>
+      </c>
+      <c r="H8" s="60">
+        <f>'📦 商品出厂底价库 (Products)'!P6</f>
+      </c>
+      <c r="I8" s="58">
+        <f>'📦 商品出厂底价库 (Products)'!J6</f>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="62">
+        <v>6</v>
+      </c>
+      <c r="B9" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!A7</f>
+      </c>
+      <c r="C9" s="63">
+        <f>'📦 商品出厂底价库 (Products)'!C7</f>
+      </c>
+      <c r="D9" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!E7</f>
+      </c>
+      <c r="E9" s="65">
+        <f>'📦 商品出厂底价库 (Products)'!N7</f>
+      </c>
+      <c r="F9" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!F7</f>
+      </c>
+      <c r="G9" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!O7</f>
+      </c>
+      <c r="H9" s="64">
+        <f>'📦 商品出厂底价库 (Products)'!P7</f>
+      </c>
+      <c r="I9" s="62">
+        <f>'📦 商品出厂底价库 (Products)'!J7</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>